<commit_message>
Track audit findings and linked corrective projects in offline v14
</commit_message>
<xml_diff>
--- a/assets/Annex_A_Domains.xlsx
+++ b/assets/Annex_A_Domains.xlsx
@@ -2388,12 +2388,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">فهرست صریح اقلام هر یک از ده حوزه در پیام کاربر</t>
+          <t xml:space="preserve">فهرست ده حوزهٔ کنترل و هشت حوزهٔ الزامات، با ادغام‌های درخواستی نسخهٔ ۱۴</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Explicit assignments in the user-provided mapping</t>
+          <t xml:space="preserve">User assignments with the version-14 requirements-domain merges</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">

</xml_diff>